<commit_message>
chore: publish Wasp Nest v3.0.1 (105)
</commit_message>
<xml_diff>
--- a/plugins/website-audit-tools/skills/audit-scoring-stinger/references/templates/website-audit-scorecard-template.xlsx
+++ b/plugins/website-audit-tools/skills/audit-scoring-stinger/references/templates/website-audit-scorecard-template.xlsx
@@ -1,28 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Scorecard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rubric" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorecard" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Tree" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue Drivers" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mission Critical" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analytics and Insight" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Technical Deployment" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Foundational Completeness" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Search Presence" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Score" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings Register" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Index" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Executive Scorecard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Rubric" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Scorecard" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Audit Tree" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Security" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Revenue Drivers" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Mission Critical" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Analytics and Insight" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Technical Deployment" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Foundational Completeness" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Search Presence" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Content Score" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Findings Register" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Evidence Index" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Config" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="Wt_security">'Rubric'!$C$17</definedName>
@@ -694,7 +694,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-18 21:18 UTC</t>
+          <t>2026-10-13 06:28 UTC</t>
         </is>
       </c>
     </row>
@@ -713,7 +713,7 @@
     <row r="16">
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>{{...}} placeholders are hydrated by audit-intake-worker-bee's four recorded answers and by audit-scoring-worker-bee at rollup time. This Cover sheet carries no formulas; it is populated by direct cell write, per the template-injection pattern in references/research/distilled-audit-scoring.md section 3.</t>
+          <t>{{...}} placeholders are hydrated by audit-intake-wasp-drone's four recorded answers and by audit-scoring-wasp-drone at rollup time. This Cover sheet carries no formulas; it is populated by direct cell write, per the template-injection pattern in references/research/distilled-audit-scoring.md section 3.</t>
         </is>
       </c>
     </row>
@@ -5839,7 +5839,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Every finding, one row each. Populated by audit-scoring-worker-bee from upstream Bees' leaf findings.</t>
+          <t>Every finding, one row each. Populated by audit-scoring-wasp-drone from upstream Drones' leaf findings.</t>
         </is>
       </c>
     </row>
@@ -6082,7 +6082,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-18 21:18 UTC</t>
+          <t>2026-10-13 06:28 UTC</t>
         </is>
       </c>
     </row>
@@ -6444,7 +6444,7 @@
         <v/>
       </c>
       <c r="D5" s="10">
-        <f>B5*C5</f>
+        <f>IF(ISNUMBER(C5),B5*C5,"N/A")</f>
         <v/>
       </c>
     </row>
@@ -6463,7 +6463,7 @@
         <v/>
       </c>
       <c r="D6" s="10">
-        <f>B6*C6</f>
+        <f>IF(ISNUMBER(C6),B6*C6,"N/A")</f>
         <v/>
       </c>
     </row>
@@ -6482,7 +6482,7 @@
         <v/>
       </c>
       <c r="D7" s="10">
-        <f>B7*C7</f>
+        <f>IF(ISNUMBER(C7),B7*C7,"N/A")</f>
         <v/>
       </c>
     </row>
@@ -6501,7 +6501,7 @@
         <v/>
       </c>
       <c r="D8" s="10">
-        <f>B8*C8</f>
+        <f>IF(ISNUMBER(C8),B8*C8,"N/A")</f>
         <v/>
       </c>
     </row>
@@ -6520,7 +6520,7 @@
         <v/>
       </c>
       <c r="D9" s="10">
-        <f>B9*C9</f>
+        <f>IF(ISNUMBER(C9),B9*C9,"N/A")</f>
         <v/>
       </c>
     </row>
@@ -6539,7 +6539,7 @@
         <v/>
       </c>
       <c r="D10" s="10">
-        <f>B10*C10</f>
+        <f>IF(ISNUMBER(C10),B10*C10,"N/A")</f>
         <v/>
       </c>
     </row>
@@ -6558,7 +6558,7 @@
         <v/>
       </c>
       <c r="D11" s="10">
-        <f>B11*C11</f>
+        <f>IF(ISNUMBER(C11),B11*C11,"N/A")</f>
         <v/>
       </c>
     </row>
@@ -6577,7 +6577,7 @@
         <v/>
       </c>
       <c r="D12" s="10">
-        <f>B12*C12</f>
+        <f>IF(ISNUMBER(C12),B12*C12,"N/A")</f>
         <v/>
       </c>
     </row>
@@ -6588,7 +6588,7 @@
         </is>
       </c>
       <c r="C14" s="11">
-        <f>SUMPRODUCT(C5:C12,CategoryWeights)/SUM(CategoryWeights)</f>
+        <f>IF(SUMPRODUCT(--ISNUMBER(C5:C12),CategoryWeights)=0,"N/A",SUMPRODUCT(--ISNUMBER(C5:C12),C5:C12,CategoryWeights)/SUMPRODUCT(--ISNUMBER(C5:C12),CategoryWeights))</f>
         <v/>
       </c>
     </row>
@@ -6632,7 +6632,7 @@
         </is>
       </c>
       <c r="C20" s="11">
-        <f>IF(C16,MIN(C14,SecurityOverrideCapPct),C14)</f>
+        <f>IF(ISNUMBER(C14),IF(C16,MIN(C14,SecurityOverrideCapPct),C14),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -6643,7 +6643,7 @@
         </is>
       </c>
       <c r="C22" s="13">
-        <f>VLOOKUP(C20,GradeTable,2,TRUE)</f>
+        <f>IF(ISNUMBER(C20),VLOOKUP(C20,GradeTable,2,TRUE),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -7870,7 +7870,7 @@
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Headers (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Headers (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E8" s="23" t="n">
@@ -7923,7 +7923,7 @@
       </c>
       <c r="D9" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Headers (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Headers (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E9" s="23" t="n">
@@ -8023,7 +8023,7 @@
         </is>
       </c>
       <c r="L11" s="11">
-        <f>IF(SUMPRODUCT(--(E7:E10&gt;0),H7:H10)=0,"N/A",SUMPRODUCT(--(E7:E10&gt;0),E7:E10,H7:H10)/(6*SUMPRODUCT(--(E7:E10&gt;0),H7:H10)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E7:E10)*(E7:E10&gt;0),H7:H10)=0,"N/A",SUMPRODUCT(ISNUMBER(E7:E10)*(E7:E10&gt;0),E7:E10,H7:H10)/(6*SUMPRODUCT(ISNUMBER(E7:E10)*(E7:E10&gt;0),H7:H10)))</f>
         <v/>
       </c>
     </row>
@@ -8057,7 +8057,7 @@
       </c>
       <c r="D13" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for TLS (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for TLS (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E13" s="23" t="n">
@@ -8110,7 +8110,7 @@
       </c>
       <c r="D14" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for TLS (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for TLS (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E14" s="23" t="n">
@@ -8163,7 +8163,7 @@
       </c>
       <c r="D15" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for TLS (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for TLS (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E15" s="23" t="n">
@@ -8263,7 +8263,7 @@
         </is>
       </c>
       <c r="L17" s="11">
-        <f>IF(SUMPRODUCT(--(E13:E16&gt;0),H13:H16)=0,"N/A",SUMPRODUCT(--(E13:E16&gt;0),E13:E16,H13:H16)/(6*SUMPRODUCT(--(E13:E16&gt;0),H13:H16)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E13:E16)*(E13:E16&gt;0),H13:H16)=0,"N/A",SUMPRODUCT(ISNUMBER(E13:E16)*(E13:E16&gt;0),E13:E16,H13:H16)/(6*SUMPRODUCT(ISNUMBER(E13:E16)*(E13:E16&gt;0),H13:H16)))</f>
         <v/>
       </c>
     </row>
@@ -8297,7 +8297,7 @@
       </c>
       <c r="D19" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for Cookies (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for Cookies (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E19" s="23" t="n">
@@ -8350,7 +8350,7 @@
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Cookies (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Cookies (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E20" s="23" t="n">
@@ -8403,7 +8403,7 @@
       </c>
       <c r="D21" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Cookies (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Cookies (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E21" s="23" t="n">
@@ -8503,7 +8503,7 @@
         </is>
       </c>
       <c r="L23" s="11">
-        <f>IF(SUMPRODUCT(--(E19:E22&gt;0),H19:H22)=0,"N/A",SUMPRODUCT(--(E19:E22&gt;0),E19:E22,H19:H22)/(6*SUMPRODUCT(--(E19:E22&gt;0),H19:H22)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E19:E22)*(E19:E22&gt;0),H19:H22)=0,"N/A",SUMPRODUCT(ISNUMBER(E19:E22)*(E19:E22&gt;0),E19:E22,H19:H22)/(6*SUMPRODUCT(ISNUMBER(E19:E22)*(E19:E22&gt;0),H19:H22)))</f>
         <v/>
       </c>
     </row>
@@ -8537,7 +8537,7 @@
       </c>
       <c r="D25" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for Content-Security-Policy (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for Content-Security-Policy (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E25" s="23" t="n">
@@ -8590,7 +8590,7 @@
       </c>
       <c r="D26" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Content-Security-Policy (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Content-Security-Policy (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E26" s="23" t="n">
@@ -8643,7 +8643,7 @@
       </c>
       <c r="D27" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Content-Security-Policy (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Content-Security-Policy (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E27" s="23" t="n">
@@ -8743,7 +8743,7 @@
         </is>
       </c>
       <c r="L29" s="11">
-        <f>IF(SUMPRODUCT(--(E25:E28&gt;0),H25:H28)=0,"N/A",SUMPRODUCT(--(E25:E28&gt;0),E25:E28,H25:H28)/(6*SUMPRODUCT(--(E25:E28&gt;0),H25:H28)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E25:E28)*(E25:E28&gt;0),H25:H28)=0,"N/A",SUMPRODUCT(ISNUMBER(E25:E28)*(E25:E28&gt;0),E25:E28,H25:H28)/(6*SUMPRODUCT(ISNUMBER(E25:E28)*(E25:E28&gt;0),H25:H28)))</f>
         <v/>
       </c>
     </row>
@@ -8777,7 +8777,7 @@
       </c>
       <c r="D31" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for Platform Exposure (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for Platform Exposure (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E31" s="23" t="n">
@@ -8830,7 +8830,7 @@
       </c>
       <c r="D32" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Platform Exposure (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Platform Exposure (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E32" s="23" t="n">
@@ -8883,7 +8883,7 @@
       </c>
       <c r="D33" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Platform Exposure (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Platform Exposure (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E33" s="23" t="n">
@@ -8983,7 +8983,7 @@
         </is>
       </c>
       <c r="L35" s="11">
-        <f>IF(SUMPRODUCT(--(E31:E34&gt;0),H31:H34)=0,"N/A",SUMPRODUCT(--(E31:E34&gt;0),E31:E34,H31:H34)/(6*SUMPRODUCT(--(E31:E34&gt;0),H31:H34)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E31:E34)*(E31:E34&gt;0),H31:H34)=0,"N/A",SUMPRODUCT(ISNUMBER(E31:E34)*(E31:E34&gt;0),E31:E34,H31:H34)/(6*SUMPRODUCT(ISNUMBER(E31:E34)*(E31:E34&gt;0),H31:H34)))</f>
         <v/>
       </c>
     </row>
@@ -9017,7 +9017,7 @@
       </c>
       <c r="D37" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for Client-Side Injection (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for Client-Side Injection (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E37" s="23" t="n">
@@ -9070,7 +9070,7 @@
       </c>
       <c r="D38" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Client-Side Injection (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Client-Side Injection (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E38" s="23" t="n">
@@ -9123,7 +9123,7 @@
       </c>
       <c r="D39" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Client-Side Injection (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Client-Side Injection (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E39" s="23" t="n">
@@ -9223,7 +9223,7 @@
         </is>
       </c>
       <c r="L41" s="11">
-        <f>IF(SUMPRODUCT(--(E37:E40&gt;0),H37:H40)=0,"N/A",SUMPRODUCT(--(E37:E40&gt;0),E37:E40,H37:H40)/(6*SUMPRODUCT(--(E37:E40&gt;0),H37:H40)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E37:E40)*(E37:E40&gt;0),H37:H40)=0,"N/A",SUMPRODUCT(ISNUMBER(E37:E40)*(E37:E40&gt;0),E37:E40,H37:H40)/(6*SUMPRODUCT(ISNUMBER(E37:E40)*(E37:E40&gt;0),H37:H40)))</f>
         <v/>
       </c>
     </row>
@@ -9257,7 +9257,7 @@
       </c>
       <c r="D43" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for Payment-Path Integrity (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for Payment-Path Integrity (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E43" s="23" t="n">
@@ -9310,7 +9310,7 @@
       </c>
       <c r="D44" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Payment-Path Integrity (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Payment-Path Integrity (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E44" s="23" t="n">
@@ -9363,7 +9363,7 @@
       </c>
       <c r="D45" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Payment-Path Integrity (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Payment-Path Integrity (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E45" s="23" t="n">
@@ -9463,7 +9463,7 @@
         </is>
       </c>
       <c r="L47" s="11">
-        <f>IF(SUMPRODUCT(--(E43:E46&gt;0),H43:H46)=0,"N/A",SUMPRODUCT(--(E43:E46&gt;0),E43:E46,H43:H46)/(6*SUMPRODUCT(--(E43:E46&gt;0),H43:H46)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E43:E46)*(E43:E46&gt;0),H43:H46)=0,"N/A",SUMPRODUCT(ISNUMBER(E43:E46)*(E43:E46&gt;0),E43:E46,H43:H46)/(6*SUMPRODUCT(ISNUMBER(E43:E46)*(E43:E46&gt;0),H43:H46)))</f>
         <v/>
       </c>
     </row>
@@ -9591,7 +9591,7 @@
         </is>
       </c>
       <c r="L55" s="25">
-        <f>IF(SUM(SubWt_security)=0,"N/A",SUMPRODUCT(L48:L54,SubWt_security)/SUM(SubWt_security))</f>
+        <f>IF(SUMPRODUCT(--ISNUMBER(L48:L54),SubWt_security)=0,"N/A",SUMPRODUCT(--ISNUMBER(L48:L54),L48:L54,SubWt_security)/SUMPRODUCT(--ISNUMBER(L48:L54),SubWt_security))</f>
         <v/>
       </c>
     </row>
@@ -9652,7 +9652,7 @@
       </c>
       <c r="D59" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for Visual UX/UI (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for Visual UX/UI (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E59" s="23" t="n">
@@ -9705,7 +9705,7 @@
       </c>
       <c r="D60" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Visual UX/UI (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Visual UX/UI (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E60" s="23" t="n">
@@ -9758,7 +9758,7 @@
       </c>
       <c r="D61" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Visual UX/UI (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Visual UX/UI (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E61" s="23" t="n">
@@ -9858,7 +9858,7 @@
         </is>
       </c>
       <c r="L63" s="11">
-        <f>IF(SUMPRODUCT(--(E59:E62&gt;0),H59:H62)=0,"N/A",SUMPRODUCT(--(E59:E62&gt;0),E59:E62,H59:H62)/(6*SUMPRODUCT(--(E59:E62&gt;0),H59:H62)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E59:E62)*(E59:E62&gt;0),H59:H62)=0,"N/A",SUMPRODUCT(ISNUMBER(E59:E62)*(E59:E62&gt;0),E59:E62,H59:H62)/(6*SUMPRODUCT(ISNUMBER(E59:E62)*(E59:E62&gt;0),H59:H62)))</f>
         <v/>
       </c>
     </row>
@@ -9892,7 +9892,7 @@
       </c>
       <c r="D65" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for Navigation &amp; User Journey (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for Navigation &amp; User Journey (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E65" s="23" t="n">
@@ -9945,7 +9945,7 @@
       </c>
       <c r="D66" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Navigation &amp; User Journey (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Navigation &amp; User Journey (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E66" s="23" t="n">
@@ -9998,7 +9998,7 @@
       </c>
       <c r="D67" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Navigation &amp; User Journey (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Navigation &amp; User Journey (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E67" s="23" t="n">
@@ -10098,7 +10098,7 @@
         </is>
       </c>
       <c r="L69" s="11">
-        <f>IF(SUMPRODUCT(--(E65:E68&gt;0),H65:H68)=0,"N/A",SUMPRODUCT(--(E65:E68&gt;0),E65:E68,H65:H68)/(6*SUMPRODUCT(--(E65:E68&gt;0),H65:H68)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E65:E68)*(E65:E68&gt;0),H65:H68)=0,"N/A",SUMPRODUCT(ISNUMBER(E65:E68)*(E65:E68&gt;0),E65:E68,H65:H68)/(6*SUMPRODUCT(ISNUMBER(E65:E68)*(E65:E68&gt;0),H65:H68)))</f>
         <v/>
       </c>
     </row>
@@ -10132,7 +10132,7 @@
       </c>
       <c r="D71" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for On-Page Copy (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for On-Page Copy (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E71" s="23" t="n">
@@ -10185,7 +10185,7 @@
       </c>
       <c r="D72" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for On-Page Copy (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for On-Page Copy (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E72" s="23" t="n">
@@ -10238,7 +10238,7 @@
       </c>
       <c r="D73" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for On-Page Copy (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for On-Page Copy (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E73" s="23" t="n">
@@ -10338,7 +10338,7 @@
         </is>
       </c>
       <c r="L75" s="11">
-        <f>IF(SUMPRODUCT(--(E71:E74&gt;0),H71:H74)=0,"N/A",SUMPRODUCT(--(E71:E74&gt;0),E71:E74,H71:H74)/(6*SUMPRODUCT(--(E71:E74&gt;0),H71:H74)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E71:E74)*(E71:E74&gt;0),H71:H74)=0,"N/A",SUMPRODUCT(ISNUMBER(E71:E74)*(E71:E74&gt;0),E71:E74,H71:H74)/(6*SUMPRODUCT(ISNUMBER(E71:E74)*(E71:E74&gt;0),H71:H74)))</f>
         <v/>
       </c>
     </row>
@@ -10402,7 +10402,7 @@
         </is>
       </c>
       <c r="L79" s="25">
-        <f>IF(SUM(SubWt_revenue)=0,"N/A",SUMPRODUCT(L76:L78,SubWt_revenue)/SUM(SubWt_revenue))</f>
+        <f>IF(SUMPRODUCT(--ISNUMBER(L76:L78),SubWt_revenue)=0,"N/A",SUMPRODUCT(--ISNUMBER(L76:L78),L76:L78,SubWt_revenue)/SUMPRODUCT(--ISNUMBER(L76:L78),SubWt_revenue))</f>
         <v/>
       </c>
     </row>
@@ -10463,7 +10463,7 @@
       </c>
       <c r="D83" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for Primary Conversion Path Integrity (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for Primary Conversion Path Integrity (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E83" s="23" t="n">
@@ -10516,7 +10516,7 @@
       </c>
       <c r="D84" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Primary Conversion Path Integrity (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Primary Conversion Path Integrity (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E84" s="23" t="n">
@@ -10569,7 +10569,7 @@
       </c>
       <c r="D85" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Primary Conversion Path Integrity (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Primary Conversion Path Integrity (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E85" s="23" t="n">
@@ -10669,7 +10669,7 @@
         </is>
       </c>
       <c r="L87" s="11">
-        <f>IF(SUMPRODUCT(--(E83:E86&gt;0),H83:H86)=0,"N/A",SUMPRODUCT(--(E83:E86&gt;0),E83:E86,H83:H86)/(6*SUMPRODUCT(--(E83:E86&gt;0),H83:H86)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E83:E86)*(E83:E86&gt;0),H83:H86)=0,"N/A",SUMPRODUCT(ISNUMBER(E83:E86)*(E83:E86&gt;0),E83:E86,H83:H86)/(6*SUMPRODUCT(ISNUMBER(E83:E86)*(E83:E86&gt;0),H83:H86)))</f>
         <v/>
       </c>
     </row>
@@ -10703,7 +10703,7 @@
       </c>
       <c r="D89" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for Core Function Reliability (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for Core Function Reliability (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E89" s="23" t="n">
@@ -10756,7 +10756,7 @@
       </c>
       <c r="D90" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Core Function Reliability (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Core Function Reliability (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E90" s="23" t="n">
@@ -10809,7 +10809,7 @@
       </c>
       <c r="D91" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Core Function Reliability (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Core Function Reliability (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E91" s="23" t="n">
@@ -10909,7 +10909,7 @@
         </is>
       </c>
       <c r="L93" s="11">
-        <f>IF(SUMPRODUCT(--(E89:E92&gt;0),H89:H92)=0,"N/A",SUMPRODUCT(--(E89:E92&gt;0),E89:E92,H89:H92)/(6*SUMPRODUCT(--(E89:E92&gt;0),H89:H92)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E89:E92)*(E89:E92&gt;0),H89:H92)=0,"N/A",SUMPRODUCT(ISNUMBER(E89:E92)*(E89:E92&gt;0),E89:E92,H89:H92)/(6*SUMPRODUCT(ISNUMBER(E89:E92)*(E89:E92&gt;0),H89:H92)))</f>
         <v/>
       </c>
     </row>
@@ -10943,7 +10943,7 @@
       </c>
       <c r="D95" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for Trust &amp; Credibility Signals (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for Trust &amp; Credibility Signals (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E95" s="23" t="n">
@@ -10996,7 +10996,7 @@
       </c>
       <c r="D96" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Trust &amp; Credibility Signals (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Trust &amp; Credibility Signals (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E96" s="23" t="n">
@@ -11049,7 +11049,7 @@
       </c>
       <c r="D97" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Trust &amp; Credibility Signals (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Trust &amp; Credibility Signals (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E97" s="23" t="n">
@@ -11149,7 +11149,7 @@
         </is>
       </c>
       <c r="L99" s="11">
-        <f>IF(SUMPRODUCT(--(E95:E98&gt;0),H95:H98)=0,"N/A",SUMPRODUCT(--(E95:E98&gt;0),E95:E98,H95:H98)/(6*SUMPRODUCT(--(E95:E98&gt;0),H95:H98)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E95:E98)*(E95:E98&gt;0),H95:H98)=0,"N/A",SUMPRODUCT(ISNUMBER(E95:E98)*(E95:E98&gt;0),E95:E98,H95:H98)/(6*SUMPRODUCT(ISNUMBER(E95:E98)*(E95:E98&gt;0),H95:H98)))</f>
         <v/>
       </c>
     </row>
@@ -11213,7 +11213,7 @@
         </is>
       </c>
       <c r="L103" s="25">
-        <f>IF(SUM(SubWt_mission)=0,"N/A",SUMPRODUCT(L100:L102,SubWt_mission)/SUM(SubWt_mission))</f>
+        <f>IF(SUMPRODUCT(--ISNUMBER(L100:L102),SubWt_mission)=0,"N/A",SUMPRODUCT(--ISNUMBER(L100:L102),L100:L102,SubWt_mission)/SUMPRODUCT(--ISNUMBER(L100:L102),SubWt_mission))</f>
         <v/>
       </c>
     </row>
@@ -11274,7 +11274,7 @@
       </c>
       <c r="D107" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for Foundational Analytics (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for Foundational Analytics (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E107" s="23" t="n">
@@ -11327,7 +11327,7 @@
       </c>
       <c r="D108" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Foundational Analytics (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Foundational Analytics (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E108" s="23" t="n">
@@ -11380,7 +11380,7 @@
       </c>
       <c r="D109" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Foundational Analytics (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Foundational Analytics (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E109" s="23" t="n">
@@ -11480,7 +11480,7 @@
         </is>
       </c>
       <c r="L111" s="11">
-        <f>IF(SUMPRODUCT(--(E107:E110&gt;0),H107:H110)=0,"N/A",SUMPRODUCT(--(E107:E110&gt;0),E107:E110,H107:H110)/(6*SUMPRODUCT(--(E107:E110&gt;0),H107:H110)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E107:E110)*(E107:E110&gt;0),H107:H110)=0,"N/A",SUMPRODUCT(ISNUMBER(E107:E110)*(E107:E110&gt;0),E107:E110,H107:H110)/(6*SUMPRODUCT(ISNUMBER(E107:E110)*(E107:E110&gt;0),H107:H110)))</f>
         <v/>
       </c>
     </row>
@@ -11514,7 +11514,7 @@
       </c>
       <c r="D113" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for Industry-Specific Analytics (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for Industry-Specific Analytics (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E113" s="23" t="n">
@@ -11567,7 +11567,7 @@
       </c>
       <c r="D114" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Industry-Specific Analytics (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Industry-Specific Analytics (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E114" s="23" t="n">
@@ -11620,7 +11620,7 @@
       </c>
       <c r="D115" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Industry-Specific Analytics (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Industry-Specific Analytics (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E115" s="23" t="n">
@@ -11720,7 +11720,7 @@
         </is>
       </c>
       <c r="L117" s="11">
-        <f>IF(SUMPRODUCT(--(E113:E116&gt;0),H113:H116)=0,"N/A",SUMPRODUCT(--(E113:E116&gt;0),E113:E116,H113:H116)/(6*SUMPRODUCT(--(E113:E116&gt;0),H113:H116)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E113:E116)*(E113:E116&gt;0),H113:H116)=0,"N/A",SUMPRODUCT(ISNUMBER(E113:E116)*(E113:E116&gt;0),E113:E116,H113:H116)/(6*SUMPRODUCT(ISNUMBER(E113:E116)*(E113:E116&gt;0),H113:H116)))</f>
         <v/>
       </c>
     </row>
@@ -11754,7 +11754,7 @@
       </c>
       <c r="D119" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for De-Anonymization (where lawful) (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for De-Anonymization (where lawful) (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E119" s="23" t="n">
@@ -11807,7 +11807,7 @@
       </c>
       <c r="D120" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for De-Anonymization (where lawful) (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for De-Anonymization (where lawful) (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E120" s="23" t="n">
@@ -11860,7 +11860,7 @@
       </c>
       <c r="D121" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for De-Anonymization (where lawful) (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for De-Anonymization (where lawful) (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E121" s="23" t="n">
@@ -11960,7 +11960,7 @@
         </is>
       </c>
       <c r="L123" s="11">
-        <f>IF(SUMPRODUCT(--(E119:E122&gt;0),H119:H122)=0,"N/A",SUMPRODUCT(--(E119:E122&gt;0),E119:E122,H119:H122)/(6*SUMPRODUCT(--(E119:E122&gt;0),H119:H122)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E119:E122)*(E119:E122&gt;0),H119:H122)=0,"N/A",SUMPRODUCT(ISNUMBER(E119:E122)*(E119:E122&gt;0),E119:E122,H119:H122)/(6*SUMPRODUCT(ISNUMBER(E119:E122)*(E119:E122&gt;0),H119:H122)))</f>
         <v/>
       </c>
     </row>
@@ -12024,7 +12024,7 @@
         </is>
       </c>
       <c r="L127" s="25">
-        <f>IF(SUM(SubWt_analytics)=0,"N/A",SUMPRODUCT(L124:L126,SubWt_analytics)/SUM(SubWt_analytics))</f>
+        <f>IF(SUMPRODUCT(--ISNUMBER(L124:L126),SubWt_analytics)=0,"N/A",SUMPRODUCT(--ISNUMBER(L124:L126),L124:L126,SubWt_analytics)/SUMPRODUCT(--ISNUMBER(L124:L126),SubWt_analytics))</f>
         <v/>
       </c>
     </row>
@@ -12085,7 +12085,7 @@
       </c>
       <c r="D131" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for CDN (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for CDN (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E131" s="23" t="n">
@@ -12138,7 +12138,7 @@
       </c>
       <c r="D132" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for CDN (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for CDN (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E132" s="23" t="n">
@@ -12191,7 +12191,7 @@
       </c>
       <c r="D133" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for CDN (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for CDN (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E133" s="23" t="n">
@@ -12291,7 +12291,7 @@
         </is>
       </c>
       <c r="L135" s="11">
-        <f>IF(SUMPRODUCT(--(E131:E134&gt;0),H131:H134)=0,"N/A",SUMPRODUCT(--(E131:E134&gt;0),E131:E134,H131:H134)/(6*SUMPRODUCT(--(E131:E134&gt;0),H131:H134)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E131:E134)*(E131:E134&gt;0),H131:H134)=0,"N/A",SUMPRODUCT(ISNUMBER(E131:E134)*(E131:E134&gt;0),E131:E134,H131:H134)/(6*SUMPRODUCT(ISNUMBER(E131:E134)*(E131:E134&gt;0),H131:H134)))</f>
         <v/>
       </c>
     </row>
@@ -12325,7 +12325,7 @@
       </c>
       <c r="D137" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for Caching Strategy (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for Caching Strategy (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E137" s="23" t="n">
@@ -12378,7 +12378,7 @@
       </c>
       <c r="D138" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Caching Strategy (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Caching Strategy (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E138" s="23" t="n">
@@ -12431,7 +12431,7 @@
       </c>
       <c r="D139" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Caching Strategy (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Caching Strategy (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E139" s="23" t="n">
@@ -12531,7 +12531,7 @@
         </is>
       </c>
       <c r="L141" s="11">
-        <f>IF(SUMPRODUCT(--(E137:E140&gt;0),H137:H140)=0,"N/A",SUMPRODUCT(--(E137:E140&gt;0),E137:E140,H137:H140)/(6*SUMPRODUCT(--(E137:E140&gt;0),H137:H140)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E137:E140)*(E137:E140&gt;0),H137:H140)=0,"N/A",SUMPRODUCT(ISNUMBER(E137:E140)*(E137:E140&gt;0),E137:E140,H137:H140)/(6*SUMPRODUCT(ISNUMBER(E137:E140)*(E137:E140&gt;0),H137:H140)))</f>
         <v/>
       </c>
     </row>
@@ -12565,7 +12565,7 @@
       </c>
       <c r="D143" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for Core Web Vitals (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for Core Web Vitals (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E143" s="23" t="n">
@@ -12618,7 +12618,7 @@
       </c>
       <c r="D144" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Core Web Vitals (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Core Web Vitals (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E144" s="23" t="n">
@@ -12671,7 +12671,7 @@
       </c>
       <c r="D145" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Core Web Vitals (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Core Web Vitals (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E145" s="23" t="n">
@@ -12771,7 +12771,7 @@
         </is>
       </c>
       <c r="L147" s="11">
-        <f>IF(SUMPRODUCT(--(E143:E146&gt;0),H143:H146)=0,"N/A",SUMPRODUCT(--(E143:E146&gt;0),E143:E146,H143:H146)/(6*SUMPRODUCT(--(E143:E146&gt;0),H143:H146)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E143:E146)*(E143:E146&gt;0),H143:H146)=0,"N/A",SUMPRODUCT(ISNUMBER(E143:E146)*(E143:E146&gt;0),E143:E146,H143:H146)/(6*SUMPRODUCT(ISNUMBER(E143:E146)*(E143:E146&gt;0),H143:H146)))</f>
         <v/>
       </c>
     </row>
@@ -12835,7 +12835,7 @@
         </is>
       </c>
       <c r="L151" s="25">
-        <f>IF(SUM(SubWt_technical)=0,"N/A",SUMPRODUCT(L148:L150,SubWt_technical)/SUM(SubWt_technical))</f>
+        <f>IF(SUMPRODUCT(--ISNUMBER(L148:L150),SubWt_technical)=0,"N/A",SUMPRODUCT(--ISNUMBER(L148:L150),L148:L150,SubWt_technical)/SUMPRODUCT(--ISNUMBER(L148:L150),SubWt_technical))</f>
         <v/>
       </c>
     </row>
@@ -12896,7 +12896,7 @@
       </c>
       <c r="D155" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for Core Pages &amp; Contact Info (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for Core Pages &amp; Contact Info (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E155" s="23" t="n">
@@ -12949,7 +12949,7 @@
       </c>
       <c r="D156" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Core Pages &amp; Contact Info (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Core Pages &amp; Contact Info (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E156" s="23" t="n">
@@ -13002,7 +13002,7 @@
       </c>
       <c r="D157" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Core Pages &amp; Contact Info (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Core Pages &amp; Contact Info (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E157" s="23" t="n">
@@ -13102,7 +13102,7 @@
         </is>
       </c>
       <c r="L159" s="11">
-        <f>IF(SUMPRODUCT(--(E155:E158&gt;0),H155:H158)=0,"N/A",SUMPRODUCT(--(E155:E158&gt;0),E155:E158,H155:H158)/(6*SUMPRODUCT(--(E155:E158&gt;0),H155:H158)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E155:E158)*(E155:E158&gt;0),H155:H158)=0,"N/A",SUMPRODUCT(ISNUMBER(E155:E158)*(E155:E158&gt;0),E155:E158,H155:H158)/(6*SUMPRODUCT(ISNUMBER(E155:E158)*(E155:E158&gt;0),H155:H158)))</f>
         <v/>
       </c>
     </row>
@@ -13136,7 +13136,7 @@
       </c>
       <c r="D161" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for Legal &amp; Policy Presence (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for Legal &amp; Policy Presence (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E161" s="23" t="n">
@@ -13189,7 +13189,7 @@
       </c>
       <c r="D162" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Legal &amp; Policy Presence (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Legal &amp; Policy Presence (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E162" s="23" t="n">
@@ -13242,7 +13242,7 @@
       </c>
       <c r="D163" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Legal &amp; Policy Presence (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Legal &amp; Policy Presence (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E163" s="23" t="n">
@@ -13342,7 +13342,7 @@
         </is>
       </c>
       <c r="L165" s="11">
-        <f>IF(SUMPRODUCT(--(E161:E164&gt;0),H161:H164)=0,"N/A",SUMPRODUCT(--(E161:E164&gt;0),E161:E164,H161:H164)/(6*SUMPRODUCT(--(E161:E164&gt;0),H161:H164)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E161:E164)*(E161:E164&gt;0),H161:H164)=0,"N/A",SUMPRODUCT(ISNUMBER(E161:E164)*(E161:E164&gt;0),E161:E164,H161:H164)/(6*SUMPRODUCT(ISNUMBER(E161:E164)*(E161:E164&gt;0),H161:H164)))</f>
         <v/>
       </c>
     </row>
@@ -13376,7 +13376,7 @@
       </c>
       <c r="D167" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for Basic Technical Hygiene (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for Basic Technical Hygiene (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E167" s="23" t="n">
@@ -13429,7 +13429,7 @@
       </c>
       <c r="D168" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Basic Technical Hygiene (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Basic Technical Hygiene (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E168" s="23" t="n">
@@ -13482,7 +13482,7 @@
       </c>
       <c r="D169" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Basic Technical Hygiene (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Basic Technical Hygiene (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E169" s="23" t="n">
@@ -13582,7 +13582,7 @@
         </is>
       </c>
       <c r="L171" s="11">
-        <f>IF(SUMPRODUCT(--(E167:E170&gt;0),H167:H170)=0,"N/A",SUMPRODUCT(--(E167:E170&gt;0),E167:E170,H167:H170)/(6*SUMPRODUCT(--(E167:E170&gt;0),H167:H170)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E167:E170)*(E167:E170&gt;0),H167:H170)=0,"N/A",SUMPRODUCT(ISNUMBER(E167:E170)*(E167:E170&gt;0),E167:E170,H167:H170)/(6*SUMPRODUCT(ISNUMBER(E167:E170)*(E167:E170&gt;0),H167:H170)))</f>
         <v/>
       </c>
     </row>
@@ -13646,7 +13646,7 @@
         </is>
       </c>
       <c r="L175" s="25">
-        <f>IF(SUM(SubWt_foundational)=0,"N/A",SUMPRODUCT(L172:L174,SubWt_foundational)/SUM(SubWt_foundational))</f>
+        <f>IF(SUMPRODUCT(--ISNUMBER(L172:L174),SubWt_foundational)=0,"N/A",SUMPRODUCT(--ISNUMBER(L172:L174),L172:L174,SubWt_foundational)/SUMPRODUCT(--ISNUMBER(L172:L174),SubWt_foundational))</f>
         <v/>
       </c>
     </row>
@@ -13707,7 +13707,7 @@
       </c>
       <c r="D179" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for Technical SEO (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for Technical SEO (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E179" s="23" t="n">
@@ -13760,7 +13760,7 @@
       </c>
       <c r="D180" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Technical SEO (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Technical SEO (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E180" s="23" t="n">
@@ -13813,7 +13813,7 @@
       </c>
       <c r="D181" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Technical SEO (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Technical SEO (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E181" s="23" t="n">
@@ -13913,7 +13913,7 @@
         </is>
       </c>
       <c r="L183" s="11">
-        <f>IF(SUMPRODUCT(--(E179:E182&gt;0),H179:H182)=0,"N/A",SUMPRODUCT(--(E179:E182&gt;0),E179:E182,H179:H182)/(6*SUMPRODUCT(--(E179:E182&gt;0),H179:H182)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E179:E182)*(E179:E182&gt;0),H179:H182)=0,"N/A",SUMPRODUCT(ISNUMBER(E179:E182)*(E179:E182&gt;0),E179:E182,H179:H182)/(6*SUMPRODUCT(ISNUMBER(E179:E182)*(E179:E182&gt;0),H179:H182)))</f>
         <v/>
       </c>
     </row>
@@ -13947,7 +13947,7 @@
       </c>
       <c r="D185" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for Technical AEO (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for Technical AEO (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E185" s="23" t="n">
@@ -14000,7 +14000,7 @@
       </c>
       <c r="D186" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Technical AEO (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Technical AEO (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E186" s="23" t="n">
@@ -14053,7 +14053,7 @@
       </c>
       <c r="D187" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Technical AEO (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Technical AEO (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E187" s="23" t="n">
@@ -14153,7 +14153,7 @@
         </is>
       </c>
       <c r="L189" s="11">
-        <f>IF(SUMPRODUCT(--(E185:E188&gt;0),H185:H188)=0,"N/A",SUMPRODUCT(--(E185:E188&gt;0),E185:E188,H185:H188)/(6*SUMPRODUCT(--(E185:E188&gt;0),H185:H188)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E185:E188)*(E185:E188&gt;0),H185:H188)=0,"N/A",SUMPRODUCT(ISNUMBER(E185:E188)*(E185:E188&gt;0),E185:E188,H185:H188)/(6*SUMPRODUCT(ISNUMBER(E185:E188)*(E185:E188&gt;0),H185:H188)))</f>
         <v/>
       </c>
     </row>
@@ -14187,7 +14187,7 @@
       </c>
       <c r="D191" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for Subjective Copy Read (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for Subjective Copy Read (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E191" s="23" t="n">
@@ -14240,7 +14240,7 @@
       </c>
       <c r="D192" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Subjective Copy Read (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Subjective Copy Read (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E192" s="23" t="n">
@@ -14293,7 +14293,7 @@
       </c>
       <c r="D193" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Subjective Copy Read (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Subjective Copy Read (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E193" s="23" t="n">
@@ -14393,7 +14393,7 @@
         </is>
       </c>
       <c r="L195" s="11">
-        <f>IF(SUMPRODUCT(--(E191:E194&gt;0),H191:H194)=0,"N/A",SUMPRODUCT(--(E191:E194&gt;0),E191:E194,H191:H194)/(6*SUMPRODUCT(--(E191:E194&gt;0),H191:H194)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E191:E194)*(E191:E194&gt;0),H191:H194)=0,"N/A",SUMPRODUCT(ISNUMBER(E191:E194)*(E191:E194&gt;0),E191:E194,H191:H194)/(6*SUMPRODUCT(ISNUMBER(E191:E194)*(E191:E194&gt;0),H191:H194)))</f>
         <v/>
       </c>
     </row>
@@ -14457,7 +14457,7 @@
         </is>
       </c>
       <c r="L199" s="25">
-        <f>IF(SUM(SubWt_search)=0,"N/A",SUMPRODUCT(L196:L198,SubWt_search)/SUM(SubWt_search))</f>
+        <f>IF(SUMPRODUCT(--ISNUMBER(L196:L198),SubWt_search)=0,"N/A",SUMPRODUCT(--ISNUMBER(L196:L198),L196:L198,SubWt_search)/SUMPRODUCT(--ISNUMBER(L196:L198),SubWt_search))</f>
         <v/>
       </c>
     </row>
@@ -14518,7 +14518,7 @@
       </c>
       <c r="D203" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for Depth (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for Depth (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E203" s="23" t="n">
@@ -14571,7 +14571,7 @@
       </c>
       <c r="D204" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Depth (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Depth (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E204" s="23" t="n">
@@ -14624,7 +14624,7 @@
       </c>
       <c r="D205" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Depth (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Depth (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E205" s="23" t="n">
@@ -14724,7 +14724,7 @@
         </is>
       </c>
       <c r="L207" s="11">
-        <f>IF(SUMPRODUCT(--(E203:E206&gt;0),H203:H206)=0,"N/A",SUMPRODUCT(--(E203:E206&gt;0),E203:E206,H203:H206)/(6*SUMPRODUCT(--(E203:E206&gt;0),H203:H206)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E203:E206)*(E203:E206&gt;0),H203:H206)=0,"N/A",SUMPRODUCT(ISNUMBER(E203:E206)*(E203:E206&gt;0),E203:E206,H203:H206)/(6*SUMPRODUCT(ISNUMBER(E203:E206)*(E203:E206&gt;0),H203:H206)))</f>
         <v/>
       </c>
     </row>
@@ -14758,7 +14758,7 @@
       </c>
       <c r="D209" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for Freshness (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for Freshness (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E209" s="23" t="n">
@@ -14811,7 +14811,7 @@
       </c>
       <c r="D210" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Freshness (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Freshness (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E210" s="23" t="n">
@@ -14864,7 +14864,7 @@
       </c>
       <c r="D211" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Freshness (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Freshness (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E211" s="23" t="n">
@@ -14964,7 +14964,7 @@
         </is>
       </c>
       <c r="L213" s="11">
-        <f>IF(SUMPRODUCT(--(E209:E212&gt;0),H209:H212)=0,"N/A",SUMPRODUCT(--(E209:E212&gt;0),E209:E212,H209:H212)/(6*SUMPRODUCT(--(E209:E212&gt;0),H209:H212)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E209:E212)*(E209:E212&gt;0),H209:H212)=0,"N/A",SUMPRODUCT(ISNUMBER(E209:E212)*(E209:E212&gt;0),E209:E212,H209:H212)/(6*SUMPRODUCT(ISNUMBER(E209:E212)*(E209:E212&gt;0),H209:H212)))</f>
         <v/>
       </c>
     </row>
@@ -14998,7 +14998,7 @@
       </c>
       <c r="D215" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 1 for Coverage (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 1 for Coverage (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E215" s="23" t="n">
@@ -15051,7 +15051,7 @@
       </c>
       <c r="D216" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 2 for Coverage (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 2 for Coverage (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E216" s="23" t="n">
@@ -15104,7 +15104,7 @@
       </c>
       <c r="D217" s="15" t="inlineStr">
         <is>
-          <t>Example leaf 3 for Coverage (illustrative placeholder - replaced by the real upstream Bee's finding at run time)</t>
+          <t>Example leaf 3 for Coverage (illustrative placeholder - replaced by the real upstream Drone's finding at run time)</t>
         </is>
       </c>
       <c r="E217" s="23" t="n">
@@ -15204,7 +15204,7 @@
         </is>
       </c>
       <c r="L219" s="11">
-        <f>IF(SUMPRODUCT(--(E215:E218&gt;0),H215:H218)=0,"N/A",SUMPRODUCT(--(E215:E218&gt;0),E215:E218,H215:H218)/(6*SUMPRODUCT(--(E215:E218&gt;0),H215:H218)))</f>
+        <f>IF(SUMPRODUCT(ISNUMBER(E215:E218)*(E215:E218&gt;0),H215:H218)=0,"N/A",SUMPRODUCT(ISNUMBER(E215:E218)*(E215:E218&gt;0),E215:E218,H215:H218)/(6*SUMPRODUCT(ISNUMBER(E215:E218)*(E215:E218&gt;0),H215:H218)))</f>
         <v/>
       </c>
     </row>
@@ -15268,7 +15268,7 @@
         </is>
       </c>
       <c r="L223" s="25">
-        <f>IF(SUM(SubWt_content)=0,"N/A",SUMPRODUCT(L220:L222,SubWt_content)/SUM(SubWt_content))</f>
+        <f>IF(SUMPRODUCT(--ISNUMBER(L220:L222),SubWt_content)=0,"N/A",SUMPRODUCT(--ISNUMBER(L220:L222),L220:L222,SubWt_content)/SUMPRODUCT(--ISNUMBER(L220:L222),SubWt_content))</f>
         <v/>
       </c>
     </row>

</xml_diff>